<commit_message>
v1.1.4: fix double text & blank pages for digital/scan_ocr_low in Step 2
- direct_engine: rasterize scan_ocr_low pages at native DPI + JPEG to drop
  the old native text layer before ScreenAI overlay (no double text when
  imported to Kho, keeps size ~1x)
- runner: enable is_digital path for Step 1 handoff segments (copy original
  PDF + merge native text for true digital pages, merge all pages not just 0)
- gitignore: add .kilo/ and temp_cleanup_*.csv
- misc: metadata export, signing/extraction steps, translations updates
</commit_message>
<xml_diff>
--- a/assets/MetaDuLieu_template.xlsx
+++ b/assets/MetaDuLieu_template.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="53" uniqueCount="49">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="56" uniqueCount="52">
   <si>
     <t>Tiêu đề hồ sơ</t>
   </si>
@@ -169,6 +169,15 @@
   </si>
   <si>
     <t>A29.110-A29.110.001-01-0001-001.pdf</t>
+  </si>
+  <si>
+    <t>Số lượng tờ</t>
+  </si>
+  <si>
+    <t>Tờ số trang số</t>
+  </si>
+  <si>
+    <t>Số thứ tự văn bản trong hồ sơ</t>
   </si>
 </sst>
 </file>
@@ -223,9 +232,9 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Hồsơ" displayName="Hồsơ" ref="A1:M2" totalsRowShown="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Hồsơ" displayName="Hồsơ" ref="A1:N2" totalsRowShown="0">
   <autoFilter ref="A1:M2"/>
-  <tableColumns count="13">
+  <tableColumns count="14">
     <tableColumn id="1" name="Tiêu đề hồ sơ"/>
     <tableColumn id="2" name="Thời hạn bảo quản"/>
     <tableColumn id="3" name="Phông"/>
@@ -239,15 +248,16 @@
     <tableColumn id="11" name="Độ mật"/>
     <tableColumn id="12" name="Đơn vị bảo quản số"/>
     <tableColumn id="13" name="Thời gian tài liệu"/>
+    <tableColumn id="14" name="Col14"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="Vănbản" displayName="Vănbản" ref="A1:T2" totalsRowShown="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="Vănbản" displayName="Vănbản" ref="A1:V2" totalsRowShown="0">
   <autoFilter ref="A1:T2"/>
-  <tableColumns count="20">
+  <tableColumns count="22">
     <tableColumn id="1" name="Tên cơ quan, tổ chức ban hành văn bản"/>
     <tableColumn id="2" name="Tên loại văn bản"/>
     <tableColumn id="3" name="Số của văn bản"/>
@@ -268,6 +278,8 @@
     <tableColumn id="18" name="Tình trạng vật lý"/>
     <tableColumn id="19" name="Tên tệp"/>
     <tableColumn id="20" name="Thời gian tài liệu"/>
+    <tableColumn id="21" name="Col21"/>
+    <tableColumn id="22" name="Col22"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -557,11 +569,11 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:M2"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ns1="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:ns2="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:ns3="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ns1:Ignorable="x14ac">
+  <dimension ref="A1:N2"/>
+  <sheetFormatPr defaultRowHeight="14.4" ns2:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:13" ht="15.15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:14" ht="15.15" customHeight="1" ns2:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -590,19 +602,22 @@
         <v>8</v>
       </c>
       <c r="J1" t="s">
+        <v>49</v>
+      </c>
+      <c r="K1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" t="s">
+      <c r="L1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" t="s">
+      <c r="M1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" t="s">
+      <c r="N1" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="2" spans="1:13" ht="15.15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:13" ht="15.15" customHeight="1" ns2:dyDescent="0.3">
       <c r="A2" t="s">
         <v>34</v>
       </c>
@@ -630,30 +645,30 @@
       <c r="I2" t="s">
         <v>41</v>
       </c>
-      <c r="J2" t="s">
+      <c r="K2" t="s">
         <v>42</v>
       </c>
-      <c r="L2" t="s">
+      <c r="M2" t="s">
         <v>43</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="0.75" bottom="0.5" header="0.5" footer="0.75"/>
   <tableParts count="1">
-    <tablePart r:id="rId1"/>
+    <tablePart ns3:id="rId1"/>
   </tableParts>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:T2"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ns1="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:ns2="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:ns3="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ns1:Ignorable="x14ac">
+  <dimension ref="A1:V2"/>
+  <sheetFormatPr defaultRowHeight="14.4" ns2:dyDescent="0.3"/>
   <cols>
     <col min="5" max="5" width="21.88671875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:22" ns2:dyDescent="0.3">
       <c r="A1" t="s">
         <v>14</v>
       </c>
@@ -714,8 +729,14 @@
       <c r="T1" t="s">
         <v>12</v>
       </c>
+      <c r="U1" t="s">
+        <v>50</v>
+      </c>
+      <c r="V1" t="s">
+        <v>51</v>
+      </c>
     </row>
-    <row r="2" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:20" ns2:dyDescent="0.3">
       <c r="A2" t="s">
         <v>44</v>
       </c>
@@ -747,7 +768,7 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="0.75" bottom="0.5" header="0.5" footer="0.75"/>
   <tableParts count="1">
-    <tablePart r:id="rId1"/>
+    <tablePart ns3:id="rId1"/>
   </tableParts>
 </worksheet>
 </file>

</xml_diff>